<commit_message>
tried an alternate method of adding regions
</commit_message>
<xml_diff>
--- a/Combined_results3.xlsx
+++ b/Combined_results3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Senior Thesis Excel Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4851007-6991-4CEC-98A6-2DFBBDC04662}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E72E9A0-F745-4379-90D7-C309A770DC85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,15 +44,6 @@
   </si>
   <si>
     <t>const</t>
-  </si>
-  <si>
-    <t>event_-9</t>
-  </si>
-  <si>
-    <t>event_-8</t>
-  </si>
-  <si>
-    <t>event_-7</t>
   </si>
   <si>
     <t>event_-6</t>
@@ -98,6 +89,15 @@
   </si>
   <si>
     <t>event_9</t>
+  </si>
+  <si>
+    <t>event_10</t>
+  </si>
+  <si>
+    <t>event_11</t>
+  </si>
+  <si>
+    <t>event_12</t>
   </si>
   <si>
     <t>ratio_lag1</t>
@@ -254,58 +254,58 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="18"/>
                 <c:pt idx="0">
-                  <c:v>4.2259828891038839E-4</c:v>
+                  <c:v>-3.7830607199496121E-3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-3.896752379256691E-4</c:v>
+                  <c:v>-3.5777993273921039E-3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.557598720444307E-3</c:v>
+                  <c:v>-1.2137754881500679E-3</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-4.589198131152882E-3</c:v>
+                  <c:v>-8.1638062385371024E-4</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-2.117569397034474E-3</c:v>
+                  <c:v>9.8915789070680091E-5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-1.4971152915593379E-3</c:v>
+                  <c:v>5.5627705587932147E-3</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-8.4959196758506092E-4</c:v>
+                  <c:v>6.9114888273656347E-5</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-1.9565448738004159E-3</c:v>
+                  <c:v>4.194009186176427E-3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3.2497048528604901E-3</c:v>
+                  <c:v>5.8580775449200428E-5</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-2.770617332444244E-3</c:v>
+                  <c:v>1.3338171726434279E-3</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2.8689804328633742E-3</c:v>
+                  <c:v>1.149376339361419E-2</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-1.2076092188229759E-3</c:v>
+                  <c:v>-7.9186122459615101E-3</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>3.7072047705640577E-4</c:v>
+                  <c:v>-3.4540050545037249E-3</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>6.9812962604581747E-3</c:v>
+                  <c:v>2.5594193822843468E-3</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>-5.4201888362079183E-3</c:v>
+                  <c:v>2.5625849864815281E-5</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-3.1309624950908512E-4</c:v>
+                  <c:v>4.4954039867825882E-4</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-1.145769904648356E-3</c:v>
+                  <c:v>-5.7463786339827586E-4</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-1.903950375971711E-3</c:v>
+                  <c:v>6.591918255759166E-5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -313,7 +313,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-325B-43E5-B3FE-10B35D9E8F83}"/>
+              <c16:uniqueId val="{00000000-5D3D-4954-B105-49809EBA4DE3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -326,11 +326,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="1676740815"/>
-        <c:axId val="1676731215"/>
+        <c:axId val="70759872"/>
+        <c:axId val="70760352"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1676740815"/>
+        <c:axId val="70759872"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -372,7 +372,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1676731215"/>
+        <c:crossAx val="70760352"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -380,7 +380,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1676731215"/>
+        <c:axId val="70760352"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -431,7 +431,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1676740815"/>
+        <c:crossAx val="70759872"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1047,23 +1047,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>130175</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>200025</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>434975</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>504825</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7E2CF2C0-EAE3-D20E-192F-FB5595A21707}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EFE3465A-6C1C-B095-E038-1120E9118824}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1397,22 +1397,22 @@
         <v>6</v>
       </c>
       <c r="B2">
-        <v>-1.12108152655874E-4</v>
+        <v>8.2299395850500782E-3</v>
       </c>
       <c r="C2">
-        <v>4.6049024114587852E-4</v>
+        <v>2.8922451221990411E-3</v>
       </c>
       <c r="D2">
-        <v>-0.24345391636727279</v>
+        <v>2.845519393180846</v>
       </c>
       <c r="E2">
-        <v>0.80765378065676774</v>
+        <v>4.4339059447146374E-3</v>
       </c>
       <c r="F2">
-        <v>-1.01465244053396E-3</v>
+        <v>2.5612433110783102E-3</v>
       </c>
       <c r="G2">
-        <v>7.9043613522221238E-4</v>
+        <v>1.389863585902185E-2</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -1420,22 +1420,22 @@
         <v>7</v>
       </c>
       <c r="B3">
-        <v>4.2259828891038839E-4</v>
+        <v>-3.7830607199496121E-3</v>
       </c>
       <c r="C3">
-        <v>2.637356716588038E-3</v>
+        <v>4.8543958407262977E-3</v>
       </c>
       <c r="D3">
-        <v>0.1602355442676355</v>
+        <v>-0.77930618846764732</v>
       </c>
       <c r="E3">
-        <v>0.87269553084562523</v>
+        <v>0.43579937010933573</v>
       </c>
       <c r="F3">
-        <v>-4.746525889986977E-3</v>
+        <v>-1.329750173447419E-2</v>
       </c>
       <c r="G3">
-        <v>5.5917224678077538E-3</v>
+        <v>5.731380294574968E-3</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
@@ -1443,22 +1443,22 @@
         <v>8</v>
       </c>
       <c r="B4">
-        <v>-3.896752379256691E-4</v>
+        <v>-3.5777993273921039E-3</v>
       </c>
       <c r="C4">
-        <v>1.08674646510546E-3</v>
+        <v>4.7986761987238039E-3</v>
       </c>
       <c r="D4">
-        <v>-0.35857051339739521</v>
+        <v>-0.74558048495616591</v>
       </c>
       <c r="E4">
-        <v>0.7199164087108163</v>
+        <v>0.45592087515646212</v>
       </c>
       <c r="F4">
-        <v>-2.5196591698585851E-3</v>
+        <v>-1.298303185036033E-2</v>
       </c>
       <c r="G4">
-        <v>1.7403086940072469E-3</v>
+        <v>5.8274331955761229E-3</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -1466,22 +1466,22 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>2.557598720444307E-3</v>
+        <v>-1.2137754881500679E-3</v>
       </c>
       <c r="C5">
-        <v>2.6792732653660219E-3</v>
+        <v>2.6299870722557672E-3</v>
       </c>
       <c r="D5">
-        <v>0.95458673570383545</v>
+        <v>-0.46151386102023723</v>
       </c>
       <c r="E5">
-        <v>0.33978672758925271</v>
+        <v>0.64442997913154088</v>
       </c>
       <c r="F5">
-        <v>-2.6936803844141229E-3</v>
+        <v>-6.3684554295773124E-3</v>
       </c>
       <c r="G5">
-        <v>7.8088778253027364E-3</v>
+        <v>3.9409044532771756E-3</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -1489,22 +1489,22 @@
         <v>10</v>
       </c>
       <c r="B6">
-        <v>-4.589198131152882E-3</v>
+        <v>-8.1638062385371024E-4</v>
       </c>
       <c r="C6">
-        <v>1.77036904634878E-3</v>
+        <v>2.2331732730977091E-3</v>
       </c>
       <c r="D6">
-        <v>-2.5922268244678541</v>
+        <v>-0.36556976285198028</v>
       </c>
       <c r="E6">
-        <v>9.5356878003700803E-3</v>
+        <v>0.71468614131647767</v>
       </c>
       <c r="F6">
-        <v>-8.0590577013410127E-3</v>
+        <v>-5.1933198103626503E-3</v>
       </c>
       <c r="G6">
-        <v>-1.1193385609647511E-3</v>
+        <v>3.5605585626552298E-3</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
@@ -1512,22 +1512,22 @@
         <v>11</v>
       </c>
       <c r="B7">
-        <v>-2.117569397034474E-3</v>
+        <v>9.8915789070680091E-5</v>
       </c>
       <c r="C7">
-        <v>1.540437553008486E-3</v>
+        <v>2.1230807066901351E-3</v>
       </c>
       <c r="D7">
-        <v>-1.374654488848863</v>
+        <v>4.659068718347923E-2</v>
       </c>
       <c r="E7">
-        <v>0.16923858708156711</v>
+        <v>0.96283945452249275</v>
       </c>
       <c r="F7">
-        <v>-5.1367715213641169E-3</v>
+        <v>-4.0622459323138302E-3</v>
       </c>
       <c r="G7">
-        <v>9.016327272951697E-4</v>
+        <v>4.2600775104551904E-3</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
@@ -1535,22 +1535,22 @@
         <v>12</v>
       </c>
       <c r="B8">
-        <v>-1.4971152915593379E-3</v>
+        <v>5.5627705587932147E-3</v>
       </c>
       <c r="C8">
-        <v>1.5258542720870279E-3</v>
+        <v>3.7280823289946928E-3</v>
       </c>
       <c r="D8">
-        <v>-0.98116531764964576</v>
+        <v>1.492126532595448</v>
       </c>
       <c r="E8">
-        <v>0.32651122420507978</v>
+        <v>0.13566597744917769</v>
       </c>
       <c r="F8">
-        <v>-4.4877347105064923E-3</v>
+        <v>-1.744136537436589E-3</v>
       </c>
       <c r="G8">
-        <v>1.493504127387817E-3</v>
+        <v>1.286967765502302E-2</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -1558,22 +1558,22 @@
         <v>13</v>
       </c>
       <c r="B9">
-        <v>-8.4959196758506092E-4</v>
+        <v>6.9114888273656347E-5</v>
       </c>
       <c r="C9">
-        <v>2.0616286976018381E-3</v>
+        <v>2.8765624319138559E-3</v>
       </c>
       <c r="D9">
-        <v>-0.4120974686534668</v>
+        <v>2.4026903607884609E-2</v>
       </c>
       <c r="E9">
-        <v>0.68026798398331523</v>
+        <v>0.98083114892281875</v>
       </c>
       <c r="F9">
-        <v>-4.8903099643788812E-3</v>
+        <v>-5.5688438775584534E-3</v>
       </c>
       <c r="G9">
-        <v>3.191126029208759E-3</v>
+        <v>5.7070736541057652E-3</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
@@ -1581,22 +1581,22 @@
         <v>14</v>
       </c>
       <c r="B10">
-        <v>-1.9565448738004159E-3</v>
+        <v>4.194009186176427E-3</v>
       </c>
       <c r="C10">
-        <v>7.7760790430644682E-4</v>
+        <v>4.6770043303695202E-3</v>
       </c>
       <c r="D10">
-        <v>-2.5161072347193669</v>
+        <v>0.89672980607333908</v>
       </c>
       <c r="E10">
-        <v>1.186590734992508E-2</v>
+        <v>0.36986311183995868</v>
       </c>
       <c r="F10">
-        <v>-3.4806283603347212E-3</v>
+        <v>-4.9727508568857036E-3</v>
       </c>
       <c r="G10">
-        <v>-4.3246138726611179E-4</v>
+        <v>1.336076922923856E-2</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -1604,22 +1604,22 @@
         <v>15</v>
       </c>
       <c r="B11">
-        <v>3.2497048528604901E-3</v>
+        <v>5.8580775449200428E-5</v>
       </c>
       <c r="C11">
-        <v>2.093466169595251E-3</v>
+        <v>2.3273444832364611E-3</v>
       </c>
       <c r="D11">
-        <v>1.552308272308401</v>
+        <v>2.5170650873194589E-2</v>
       </c>
       <c r="E11">
-        <v>0.1205884795125569</v>
+        <v>0.97991884674678864</v>
       </c>
       <c r="F11">
-        <v>-8.5341344239922307E-4</v>
+        <v>-4.5029305913122462E-3</v>
       </c>
       <c r="G11">
-        <v>7.3528231481202024E-3</v>
+        <v>4.620092142210647E-3</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
@@ -1627,22 +1627,22 @@
         <v>16</v>
       </c>
       <c r="B12">
-        <v>-2.770617332444244E-3</v>
+        <v>1.3338171726434279E-3</v>
       </c>
       <c r="C12">
-        <v>2.6650329002196349E-3</v>
+        <v>2.2124837672522742E-3</v>
       </c>
       <c r="D12">
-        <v>-1.0396184348102819</v>
+        <v>0.60285964235566858</v>
       </c>
       <c r="E12">
-        <v>0.29851720873709209</v>
+        <v>0.54660206576021775</v>
       </c>
       <c r="F12">
-        <v>-7.9939858344890563E-3</v>
+        <v>-3.0025713275505278E-3</v>
       </c>
       <c r="G12">
-        <v>2.4527511696005679E-3</v>
+        <v>5.670205672837385E-3</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
@@ -1650,22 +1650,22 @@
         <v>17</v>
       </c>
       <c r="B13">
-        <v>2.8689804328633742E-3</v>
+        <v>1.149376339361419E-2</v>
       </c>
       <c r="C13">
-        <v>2.4738691329366418E-3</v>
+        <v>8.2915062548400646E-3</v>
       </c>
       <c r="D13">
-        <v>1.1597139050996239</v>
+        <v>1.3862093376465641</v>
       </c>
       <c r="E13">
-        <v>0.24616530690369881</v>
+        <v>0.16568299104798331</v>
       </c>
       <c r="F13">
-        <v>-1.979713970157775E-3</v>
+        <v>-4.7572902434609276E-3</v>
       </c>
       <c r="G13">
-        <v>7.7176748358845229E-3</v>
+        <v>2.77448170306893E-2</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
@@ -1673,22 +1673,22 @@
         <v>18</v>
       </c>
       <c r="B14">
-        <v>-1.2076092188229759E-3</v>
+        <v>-7.9186122459615101E-3</v>
       </c>
       <c r="C14">
-        <v>1.93732921881167E-3</v>
+        <v>5.2167115555879677E-3</v>
       </c>
       <c r="D14">
-        <v>-0.62333712158830001</v>
+        <v>-1.517931777822632</v>
       </c>
       <c r="E14">
-        <v>0.53306300850782495</v>
+        <v>0.1290315979552604</v>
       </c>
       <c r="F14">
-        <v>-5.0047047138909676E-3</v>
+        <v>-1.814317901264785E-2</v>
       </c>
       <c r="G14">
-        <v>2.5894862762450149E-3</v>
+        <v>2.3059545207248268E-3</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
@@ -1696,22 +1696,22 @@
         <v>19</v>
       </c>
       <c r="B15">
-        <v>3.7072047705640577E-4</v>
+        <v>-3.4540050545037249E-3</v>
       </c>
       <c r="C15">
-        <v>2.4566595984301881E-3</v>
+        <v>5.5720710132543191E-3</v>
       </c>
       <c r="D15">
-        <v>0.15090429186579091</v>
+        <v>-0.61987814697401777</v>
       </c>
       <c r="E15">
-        <v>0.88005121484168125</v>
+        <v>0.53533801409171444</v>
       </c>
       <c r="F15">
-        <v>-4.4442438581413944E-3</v>
+        <v>-1.4375063559781799E-2</v>
       </c>
       <c r="G15">
-        <v>5.185684812254206E-3</v>
+        <v>7.4670534507743471E-3</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
@@ -1719,22 +1719,22 @@
         <v>20</v>
       </c>
       <c r="B16">
-        <v>6.9812962604581747E-3</v>
+        <v>2.5594193822843468E-3</v>
       </c>
       <c r="C16">
-        <v>6.3735992709165303E-3</v>
+        <v>2.1494834460246619E-3</v>
       </c>
       <c r="D16">
-        <v>1.0953459675939521</v>
+        <v>1.1907136977574011</v>
       </c>
       <c r="E16">
-        <v>0.27336509614670718</v>
+        <v>0.23376599867732861</v>
       </c>
       <c r="F16">
-        <v>-5.510728762428971E-3</v>
+        <v>-1.6534907572890369E-3</v>
       </c>
       <c r="G16">
-        <v>1.9473321283345321E-2</v>
+        <v>6.7723295218577303E-3</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
@@ -1742,22 +1742,22 @@
         <v>21</v>
       </c>
       <c r="B17">
-        <v>-5.4201888362079183E-3</v>
+        <v>2.5625849864815281E-5</v>
       </c>
       <c r="C17">
-        <v>2.9331048149129342E-3</v>
+        <v>2.0879959107363748E-3</v>
       </c>
       <c r="D17">
-        <v>-1.847935610295881</v>
+        <v>1.2272940637981331E-2</v>
       </c>
       <c r="E17">
-        <v>6.4611658243060532E-2</v>
+        <v>0.99020785597365468</v>
       </c>
       <c r="F17">
-        <v>-1.1168968636318289E-2</v>
+        <v>-4.0667709350453891E-3</v>
       </c>
       <c r="G17">
-        <v>3.2859096390245278E-4</v>
+        <v>4.1180226347750197E-3</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
@@ -1765,22 +1765,22 @@
         <v>22</v>
       </c>
       <c r="B18">
-        <v>-3.1309624950908512E-4</v>
+        <v>4.4954039867825882E-4</v>
       </c>
       <c r="C18">
-        <v>6.5750539834544914E-4</v>
+        <v>1.751476702107533E-3</v>
       </c>
       <c r="D18">
-        <v>-0.47618810476227652</v>
+        <v>0.25666364738813352</v>
       </c>
       <c r="E18">
-        <v>0.63394037319600005</v>
+        <v>0.79743843678979931</v>
       </c>
       <c r="F18">
-        <v>-1.601783149906827E-3</v>
+        <v>-2.9832908572134951E-3</v>
       </c>
       <c r="G18">
-        <v>9.755906508886568E-4</v>
+        <v>3.8823716545700131E-3</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
@@ -1788,22 +1788,22 @@
         <v>23</v>
       </c>
       <c r="B19">
-        <v>-1.145769904648356E-3</v>
+        <v>-5.7463786339827586E-4</v>
       </c>
       <c r="C19">
-        <v>3.5983029361454571E-4</v>
+        <v>2.2448957317544962E-3</v>
       </c>
       <c r="D19">
-        <v>-3.1841952303096481</v>
+        <v>-0.25597530222446818</v>
       </c>
       <c r="E19">
-        <v>1.4515707581715181E-3</v>
+        <v>0.79796990808853663</v>
       </c>
       <c r="F19">
-        <v>-1.8510243206793389E-3</v>
+        <v>-4.9745526466847788E-3</v>
       </c>
       <c r="G19">
-        <v>-4.4051548861737399E-4</v>
+        <v>3.8252769198882271E-3</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
@@ -1811,22 +1811,22 @@
         <v>24</v>
       </c>
       <c r="B20">
-        <v>-1.903950375971711E-3</v>
+        <v>6.591918255759166E-5</v>
       </c>
       <c r="C20">
-        <v>1.117365091051641E-3</v>
+        <v>2.3338826342212118E-3</v>
       </c>
       <c r="D20">
-        <v>-1.7039644349187191</v>
+        <v>2.824442908612158E-2</v>
       </c>
       <c r="E20">
-        <v>8.8387731779073303E-2</v>
+        <v>0.97746720205821847</v>
       </c>
       <c r="F20">
-        <v>-4.0939457120152453E-3</v>
+        <v>-4.5084067246594526E-3</v>
       </c>
       <c r="G20">
-        <v>2.8604496007182239E-4</v>
+        <v>4.6402450897746359E-3</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
@@ -1834,22 +1834,22 @@
         <v>25</v>
       </c>
       <c r="B21">
-        <v>0.31582108344735288</v>
+        <v>0.48111662819587708</v>
       </c>
       <c r="C21">
-        <v>8.8921539175626396E-2</v>
+        <v>7.5670935776929418E-2</v>
       </c>
       <c r="D21">
-        <v>3.5516825999107331</v>
+        <v>6.3580108169160514</v>
       </c>
       <c r="E21">
-        <v>3.8277629432283827E-4</v>
+        <v>2.0438308215913381E-10</v>
       </c>
       <c r="F21">
-        <v>0.14153806921325771</v>
+        <v>0.332804319396652</v>
       </c>
       <c r="G21">
-        <v>0.49010409768144808</v>
+        <v>0.62942893699510216</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
@@ -1857,22 +1857,22 @@
         <v>26</v>
       </c>
       <c r="B22">
-        <v>0.1146033035213822</v>
+        <v>0.43999984485078969</v>
       </c>
       <c r="C22">
-        <v>7.731389078761873E-2</v>
+        <v>5.7339874686766122E-2</v>
       </c>
       <c r="D22">
-        <v>1.4823119410223129</v>
+        <v>7.6735403984470247</v>
       </c>
       <c r="E22">
-        <v>0.13825731247332601</v>
+        <v>1.673128045636009E-14</v>
       </c>
       <c r="F22">
-        <v>-3.692913792701355E-2</v>
+        <v>0.32761575558668832</v>
       </c>
       <c r="G22">
-        <v>0.26613574496977799</v>
+        <v>0.55238393411489128</v>
       </c>
     </row>
   </sheetData>
@@ -1911,22 +1911,22 @@
         <v>6</v>
       </c>
       <c r="B2">
-        <v>-2.344797385380471E-4</v>
+        <v>1.2574450729957319E-2</v>
       </c>
       <c r="C2">
-        <v>7.1675918901620305E-4</v>
+        <v>4.6697885777947958E-3</v>
       </c>
       <c r="D2">
-        <v>-0.32713879658785439</v>
+        <v>2.6927237754937772</v>
       </c>
       <c r="E2">
-        <v>0.74356290930140201</v>
+        <v>7.0870958182675664E-3</v>
       </c>
       <c r="F2">
-        <v>-1.6393019345979419E-3</v>
+        <v>3.421833302062997E-3</v>
       </c>
       <c r="G2">
-        <v>1.1703424575218481E-3</v>
+        <v>2.172706815785164E-2</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -1934,22 +1934,22 @@
         <v>7</v>
       </c>
       <c r="B3">
-        <v>1.560959609230422E-3</v>
+        <v>-5.025636334073269E-3</v>
       </c>
       <c r="C3">
-        <v>3.3509367425413588E-3</v>
+        <v>6.6426925226255413E-3</v>
       </c>
       <c r="D3">
-        <v>0.46582783536718941</v>
+        <v>-0.75656615400389982</v>
       </c>
       <c r="E3">
-        <v>0.64133873910843286</v>
+        <v>0.44930982510402251</v>
       </c>
       <c r="F3">
-        <v>-5.0067557206226092E-3</v>
+        <v>-1.8045074438792851E-2</v>
       </c>
       <c r="G3">
-        <v>8.1286749390834523E-3</v>
+        <v>7.9938017706463107E-3</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
@@ -1957,22 +1957,22 @@
         <v>8</v>
       </c>
       <c r="B4">
-        <v>2.3975716269531402E-5</v>
+        <v>-5.4464663042648326E-3</v>
       </c>
       <c r="C4">
-        <v>1.087369972570196E-3</v>
+        <v>6.3143699310144576E-3</v>
       </c>
       <c r="D4">
-        <v>2.2049271981329822E-2</v>
+        <v>-0.86255103260790589</v>
       </c>
       <c r="E4">
-        <v>0.9824086517194921</v>
+        <v>0.38838436317436448</v>
       </c>
       <c r="F4">
-        <v>-2.107230267838359E-3</v>
+        <v>-1.7822403954115839E-2</v>
       </c>
       <c r="G4">
-        <v>2.1551817003774218E-3</v>
+        <v>6.9294713455861721E-3</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -1980,22 +1980,22 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>3.5390615632729799E-3</v>
+        <v>-2.1410386335775108E-3</v>
       </c>
       <c r="C5">
-        <v>3.0882679876616239E-3</v>
+        <v>3.5903656908214572E-3</v>
       </c>
       <c r="D5">
-        <v>1.1459697077495821</v>
+        <v>-0.5963288472399737</v>
       </c>
       <c r="E5">
-        <v>0.25180768624740713</v>
+        <v>0.55095556340941942</v>
       </c>
       <c r="F5">
-        <v>-2.5138324671517909E-3</v>
+        <v>-9.178026078915838E-3</v>
       </c>
       <c r="G5">
-        <v>9.5919555936977499E-3</v>
+        <v>4.8959488117608146E-3</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -2003,22 +2003,22 @@
         <v>10</v>
       </c>
       <c r="B6">
-        <v>-5.1263051688272589E-3</v>
+        <v>-2.568734344608498E-3</v>
       </c>
       <c r="C6">
-        <v>2.9411838556506532E-3</v>
+        <v>3.3511593369729082E-3</v>
       </c>
       <c r="D6">
-        <v>-1.742939381017788</v>
+        <v>-0.76652110100166937</v>
       </c>
       <c r="E6">
-        <v>8.1344204128909553E-2</v>
+        <v>0.44336630137478472</v>
       </c>
       <c r="F6">
-        <v>-1.089091959781319E-2</v>
+        <v>-9.1368859515305236E-3</v>
       </c>
       <c r="G6">
-        <v>6.3830926015867335E-4</v>
+        <v>3.9994172623135276E-3</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
@@ -2026,22 +2026,22 @@
         <v>11</v>
       </c>
       <c r="B7">
-        <v>-2.059986651720636E-3</v>
+        <v>-6.0576831369959019E-4</v>
       </c>
       <c r="C7">
-        <v>2.3427430451026521E-3</v>
+        <v>2.784279624876187E-3</v>
       </c>
       <c r="D7">
-        <v>-0.87930541765000692</v>
+        <v>-0.21756734068207251</v>
       </c>
       <c r="E7">
-        <v>0.37923569921035571</v>
+        <v>0.82776623326304477</v>
       </c>
       <c r="F7">
-        <v>-6.6516786451535298E-3</v>
+        <v>-6.0628561013456074E-3</v>
       </c>
       <c r="G7">
-        <v>2.531705341712257E-3</v>
+        <v>4.851319473946427E-3</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
@@ -2049,22 +2049,22 @@
         <v>12</v>
       </c>
       <c r="B8">
-        <v>-6.3156440760738105E-4</v>
+        <v>6.5696313442708959E-3</v>
       </c>
       <c r="C8">
-        <v>2.5253178378248742E-3</v>
+        <v>5.4361656532149489E-3</v>
       </c>
       <c r="D8">
-        <v>-0.25009303706157038</v>
+        <v>1.2085046268569131</v>
       </c>
       <c r="E8">
-        <v>0.80251540054020887</v>
+        <v>0.22685321715408471</v>
       </c>
       <c r="F8">
-        <v>-5.5810964192606954E-3</v>
+        <v>-4.0850575500240606E-3</v>
       </c>
       <c r="G8">
-        <v>4.317967604045932E-3</v>
+        <v>1.7224320238565849E-2</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -2072,22 +2072,22 @@
         <v>13</v>
       </c>
       <c r="B9">
-        <v>-5.8418002621552032E-4</v>
+        <v>-2.7493059054289099E-3</v>
       </c>
       <c r="C9">
-        <v>3.2872723305051722E-3</v>
+        <v>3.7256656131935051E-3</v>
       </c>
       <c r="D9">
-        <v>-0.177709653317876</v>
+        <v>-0.73793683890817718</v>
       </c>
       <c r="E9">
-        <v>0.85895100367420352</v>
+        <v>0.46055283150741672</v>
       </c>
       <c r="F9">
-        <v>-7.0271154013807069E-3</v>
+        <v>-1.0051476325727509E-2</v>
       </c>
       <c r="G9">
-        <v>5.8587553489496663E-3</v>
+        <v>4.5528645148696948E-3</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
@@ -2095,22 +2095,22 @@
         <v>14</v>
       </c>
       <c r="B10">
-        <v>-1.7988950808541029E-3</v>
+        <v>4.7770747177000167E-3</v>
       </c>
       <c r="C10">
-        <v>9.9196131324816913E-4</v>
+        <v>4.3660949943577984E-3</v>
       </c>
       <c r="D10">
-        <v>-1.8134730224141871</v>
+        <v>1.094129817118803</v>
       </c>
       <c r="E10">
-        <v>6.9758895838648111E-2</v>
+        <v>0.27389804685172098</v>
       </c>
       <c r="F10">
-        <v>-3.74310352887757E-3</v>
+        <v>-3.7803142243218791E-3</v>
       </c>
       <c r="G10">
-        <v>1.4531336716936311E-4</v>
+        <v>1.333446365972191E-2</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -2118,22 +2118,22 @@
         <v>15</v>
       </c>
       <c r="B11">
-        <v>5.3260510483540049E-3</v>
+        <v>-1.630725295981687E-3</v>
       </c>
       <c r="C11">
-        <v>3.2961084954701309E-3</v>
+        <v>2.922484147407698E-3</v>
       </c>
       <c r="D11">
-        <v>1.6158603564396139</v>
+        <v>-0.55799286282807481</v>
       </c>
       <c r="E11">
-        <v>0.10612450850679971</v>
+        <v>0.57684925783046492</v>
       </c>
       <c r="F11">
-        <v>-1.134202891903956E-3</v>
+        <v>-7.3586889702900206E-3</v>
       </c>
       <c r="G11">
-        <v>1.1786304988611969E-2</v>
+        <v>4.0972383783266474E-3</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
@@ -2141,22 +2141,22 @@
         <v>16</v>
       </c>
       <c r="B12">
-        <v>-6.2183206034102916E-3</v>
+        <v>2.386964273794201E-5</v>
       </c>
       <c r="C12">
-        <v>3.760793484629061E-3</v>
+        <v>2.2437075210526621E-3</v>
       </c>
       <c r="D12">
-        <v>-1.6534597363097761</v>
+        <v>1.063848229502894E-2</v>
       </c>
       <c r="E12">
-        <v>9.8237334035155319E-2</v>
+        <v>0.99151187933716145</v>
       </c>
       <c r="F12">
-        <v>-1.3589340386576139E-2</v>
+        <v>-4.3737162903669212E-3</v>
       </c>
       <c r="G12">
-        <v>1.152699179755556E-3</v>
+        <v>4.4214555758428052E-3</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
@@ -2164,22 +2164,22 @@
         <v>17</v>
       </c>
       <c r="B13">
-        <v>3.858463109282775E-3</v>
+        <v>1.590140544933618E-2</v>
       </c>
       <c r="C13">
-        <v>2.1629684225041418E-3</v>
+        <v>1.1144406117155741E-2</v>
       </c>
       <c r="D13">
-        <v>1.7838739896238069</v>
+        <v>1.42685085972033</v>
       </c>
       <c r="E13">
-        <v>7.444414328561158E-2</v>
+        <v>0.15362288765354171</v>
       </c>
       <c r="F13">
-        <v>-3.8087709852275761E-4</v>
+        <v>-5.9412291693769458E-3</v>
       </c>
       <c r="G13">
-        <v>8.0978033170883076E-3</v>
+        <v>3.7744040068049309E-2</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
@@ -2187,22 +2187,22 @@
         <v>18</v>
       </c>
       <c r="B14">
-        <v>-2.2098822644117419E-3</v>
+        <v>-1.0181089244814151E-2</v>
       </c>
       <c r="C14">
-        <v>2.5405844656499251E-3</v>
+        <v>6.4226906220311531E-3</v>
       </c>
       <c r="D14">
-        <v>-0.86983223517680464</v>
+        <v>-1.5851750993409079</v>
       </c>
       <c r="E14">
-        <v>0.38439209250526918</v>
+        <v>0.1129265563933915</v>
       </c>
       <c r="F14">
-        <v>-7.1893363167675334E-3</v>
+        <v>-2.2769331547838369E-2</v>
       </c>
       <c r="G14">
-        <v>2.7695717879440492E-3</v>
+        <v>2.4071530582100639E-3</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
@@ -2210,22 +2210,22 @@
         <v>19</v>
       </c>
       <c r="B15">
-        <v>-5.6227069073396321E-4</v>
+        <v>-5.5507522356168619E-3</v>
       </c>
       <c r="C15">
-        <v>2.3577569891480611E-3</v>
+        <v>6.9764047832583708E-3</v>
       </c>
       <c r="D15">
-        <v>-0.2384769479305546</v>
+        <v>-0.79564652683819048</v>
       </c>
       <c r="E15">
-        <v>0.81151119254560045</v>
+        <v>0.42623751543871258</v>
       </c>
       <c r="F15">
-        <v>-5.1833894737617573E-3</v>
+        <v>-1.9224254352376229E-2</v>
       </c>
       <c r="G15">
-        <v>4.0588480922938309E-3</v>
+        <v>8.1227498811425065E-3</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
@@ -2233,22 +2233,22 @@
         <v>20</v>
       </c>
       <c r="B16">
-        <v>9.9873178177160623E-3</v>
+        <v>2.4545383171785898E-3</v>
       </c>
       <c r="C16">
-        <v>8.8593509248053991E-3</v>
+        <v>2.8483104612856301E-3</v>
       </c>
       <c r="D16">
-        <v>1.127319360355447</v>
+        <v>0.8617523793634122</v>
       </c>
       <c r="E16">
-        <v>0.25960747970176101</v>
+        <v>0.38882379505979853</v>
       </c>
       <c r="F16">
-        <v>-7.3766909213041406E-3</v>
+        <v>-3.128047603729913E-3</v>
       </c>
       <c r="G16">
-        <v>2.735132655673626E-2</v>
+        <v>8.0371242380870931E-3</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
@@ -2256,22 +2256,22 @@
         <v>21</v>
       </c>
       <c r="B17">
-        <v>-7.2544662521249166E-3</v>
+        <v>-2.0496975080634E-4</v>
       </c>
       <c r="C17">
-        <v>3.9953363053878586E-3</v>
+        <v>2.8139659305858318E-3</v>
       </c>
       <c r="D17">
-        <v>-1.8157335697478081</v>
+        <v>-7.2840167884928128E-2</v>
       </c>
       <c r="E17">
-        <v>6.9411251889833672E-2</v>
+        <v>0.94193330648564244</v>
       </c>
       <c r="F17">
-        <v>-1.508518151681044E-2</v>
+        <v>-5.7202416284773084E-3</v>
       </c>
       <c r="G17">
-        <v>5.7624901256061057E-4</v>
+        <v>5.3103021268646284E-3</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
@@ -2279,22 +2279,22 @@
         <v>22</v>
       </c>
       <c r="B18">
-        <v>-3.1564953287813548E-4</v>
+        <v>1.4640410754743549E-4</v>
       </c>
       <c r="C18">
-        <v>1.5777196599897679E-3</v>
+        <v>2.2607736537296418E-3</v>
       </c>
       <c r="D18">
-        <v>-0.20006693260080349</v>
+        <v>6.475841016012808E-2</v>
       </c>
       <c r="E18">
-        <v>0.84142823446313764</v>
+        <v>0.94836635579058304</v>
       </c>
       <c r="F18">
-        <v>-3.4079232441588609E-3</v>
+        <v>-4.2846308309596893E-3</v>
       </c>
       <c r="G18">
-        <v>2.7766241784025901E-3</v>
+        <v>4.5774390460545603E-3</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
@@ -2302,22 +2302,22 @@
         <v>23</v>
       </c>
       <c r="B19">
-        <v>2.5440051656092219E-5</v>
+        <v>-2.4619187821154562E-3</v>
       </c>
       <c r="C19">
-        <v>9.351114185054372E-4</v>
+        <v>2.9195839242532628E-3</v>
       </c>
       <c r="D19">
-        <v>2.720536949142633E-2</v>
+        <v>-0.84324302571474707</v>
       </c>
       <c r="E19">
-        <v>0.97829593305775286</v>
+        <v>0.39909253976574732</v>
       </c>
       <c r="F19">
-        <v>-1.807344650146727E-3</v>
+        <v>-8.1841981234939687E-3</v>
       </c>
       <c r="G19">
-        <v>1.858224753458911E-3</v>
+        <v>3.2603605592630559E-3</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
@@ -2325,22 +2325,22 @@
         <v>24</v>
       </c>
       <c r="B20">
-        <v>-1.8109217608655731E-3</v>
+        <v>-1.784046504221978E-3</v>
       </c>
       <c r="C20">
-        <v>4.7623594945249941E-4</v>
+        <v>3.8119608102006931E-3</v>
       </c>
       <c r="D20">
-        <v>-3.8025725755216171</v>
+        <v>-0.46801281362807368</v>
       </c>
       <c r="E20">
-        <v>1.432012967571539E-4</v>
+        <v>0.63977542643825469</v>
       </c>
       <c r="F20">
-        <v>-2.74432706993571E-3</v>
+        <v>-9.2553524026934599E-3</v>
       </c>
       <c r="G20">
-        <v>-8.7751645179543663E-4</v>
+        <v>5.6872593942495064E-3</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
@@ -2348,22 +2348,22 @@
         <v>25</v>
       </c>
       <c r="B21">
-        <v>0.36009813758540671</v>
+        <v>0.47130800624736219</v>
       </c>
       <c r="C21">
-        <v>9.4247207162561158E-2</v>
+        <v>7.8935694298025091E-2</v>
       </c>
       <c r="D21">
-        <v>3.8207831131196892</v>
+        <v>5.9707843256299071</v>
       </c>
       <c r="E21">
-        <v>1.3302860069333561E-4</v>
+        <v>2.3611570598453568E-9</v>
       </c>
       <c r="F21">
-        <v>0.17537700590330141</v>
+        <v>0.31659688832856941</v>
       </c>
       <c r="G21">
-        <v>0.54481926926751201</v>
+        <v>0.62601912416615513</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
@@ -2371,22 +2371,22 @@
         <v>26</v>
       </c>
       <c r="B22">
-        <v>0.11769813277561771</v>
+        <v>0.4371789258498916</v>
       </c>
       <c r="C22">
-        <v>7.7254517106674081E-2</v>
+        <v>5.6265384840226203E-2</v>
       </c>
       <c r="D22">
-        <v>1.5235113386716079</v>
+        <v>7.7699446487627366</v>
       </c>
       <c r="E22">
-        <v>0.12763082612292961</v>
+        <v>7.852043090408596E-15</v>
       </c>
       <c r="F22">
-        <v>-3.3717938396496991E-2</v>
+        <v>0.3269007979867623</v>
       </c>
       <c r="G22">
-        <v>0.26911420394773239</v>
+        <v>0.54745705371302089</v>
       </c>
     </row>
   </sheetData>
@@ -2424,22 +2424,22 @@
         <v>6</v>
       </c>
       <c r="B2">
-        <v>-2.249938485353773E-5</v>
+        <v>2.4184071050008262E-3</v>
       </c>
       <c r="C2">
-        <v>2.7049300080476431E-4</v>
+        <v>1.004050129544789E-3</v>
       </c>
       <c r="D2">
-        <v>-8.3179175751676007E-2</v>
+        <v>2.40865175337139</v>
       </c>
       <c r="E2">
-        <v>0.93370907069335884</v>
+        <v>1.6011568107094969E-2</v>
       </c>
       <c r="F2">
-        <v>-5.5265592450103951E-4</v>
+        <v>4.5050501242026439E-4</v>
       </c>
       <c r="G2">
-        <v>5.0765715479396401E-4</v>
+        <v>4.3863091975813867E-3</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -2447,22 +2447,22 @@
         <v>7</v>
       </c>
       <c r="B3">
-        <v>-5.6716551264575691E-4</v>
+        <v>-6.6467194546237325E-4</v>
       </c>
       <c r="C3">
-        <v>7.1891369611618635E-4</v>
+        <v>1.628590659037271E-3</v>
       </c>
       <c r="D3">
-        <v>-0.78892016623104533</v>
+        <v>-0.4081270770982372</v>
       </c>
       <c r="E3">
-        <v>0.43015866835055122</v>
+        <v>0.68318038193774133</v>
       </c>
       <c r="F3">
-        <v>-1.9762104650260549E-3</v>
+        <v>-3.856650982733776E-3</v>
       </c>
       <c r="G3">
-        <v>8.4187943973454134E-4</v>
+        <v>2.527307091809029E-3</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
@@ -2470,22 +2470,22 @@
         <v>8</v>
       </c>
       <c r="B4">
-        <v>-7.12779847370613E-4</v>
+        <v>-1.2490951160405829E-3</v>
       </c>
       <c r="C4">
-        <v>3.7132704027812108E-4</v>
+        <v>1.503989683463772E-3</v>
       </c>
       <c r="D4">
-        <v>-1.919547380219728</v>
+        <v>-0.83052106658328084</v>
       </c>
       <c r="E4">
-        <v>5.4915096072848807E-2</v>
+        <v>0.40624424207075233</v>
       </c>
       <c r="F4">
-        <v>-1.440567472801585E-3</v>
+        <v>-4.1968607287493727E-3</v>
       </c>
       <c r="G4">
-        <v>1.5007778060358481E-5</v>
+        <v>1.698670496668207E-3</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -2493,22 +2493,22 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>5.2186410206855416E-4</v>
+        <v>-4.7762413838108812E-4</v>
       </c>
       <c r="C5">
-        <v>9.6656321430114859E-4</v>
+        <v>1.0945342939858509E-3</v>
       </c>
       <c r="D5">
-        <v>0.53991719770328328</v>
+        <v>-0.43637201776636347</v>
       </c>
       <c r="E5">
-        <v>0.58925413715292674</v>
+        <v>0.66256683777072545</v>
       </c>
       <c r="F5">
-        <v>-1.372564986742967E-3</v>
+        <v>-2.6228719344373319E-3</v>
       </c>
       <c r="G5">
-        <v>2.416293190880076E-3</v>
+        <v>1.6676236576751559E-3</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -2516,22 +2516,22 @@
         <v>10</v>
       </c>
       <c r="B6">
-        <v>-1.8456872962901831E-3</v>
+        <v>-2.401613576437558E-4</v>
       </c>
       <c r="C6">
-        <v>6.1948927054912074E-4</v>
+        <v>1.2183145630922569E-3</v>
       </c>
       <c r="D6">
-        <v>-2.9793692708416879</v>
+        <v>-0.19712590238943861</v>
       </c>
       <c r="E6">
-        <v>2.8884245233177599E-3</v>
+        <v>0.8437290139311231</v>
       </c>
       <c r="F6">
-        <v>-3.0598639553754488E-3</v>
+        <v>-2.6280140231452298E-3</v>
       </c>
       <c r="G6">
-        <v>-6.3151063720491714E-4</v>
+        <v>2.1476913078577191E-3</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
@@ -2539,22 +2539,22 @@
         <v>11</v>
       </c>
       <c r="B7">
-        <v>-1.306095774792981E-3</v>
+        <v>3.7712562704188962E-4</v>
       </c>
       <c r="C7">
-        <v>2.9713381135861152E-4</v>
+        <v>8.5963494354203743E-4</v>
       </c>
       <c r="D7">
-        <v>-4.395648441424429</v>
+        <v>0.43870439408614798</v>
       </c>
       <c r="E7">
-        <v>1.104425587091297E-5</v>
+        <v>0.66087574276609951</v>
       </c>
       <c r="F7">
-        <v>-1.8884673436449779E-3</v>
+        <v>-1.307727902152627E-3</v>
       </c>
       <c r="G7">
-        <v>-7.2372420594098402E-4</v>
+        <v>2.061979156236406E-3</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
@@ -2562,22 +2562,22 @@
         <v>12</v>
       </c>
       <c r="B8">
-        <v>-9.1806854488293561E-4</v>
+        <v>2.0498170654343079E-3</v>
       </c>
       <c r="C8">
-        <v>4.6604004980566819E-4</v>
+        <v>1.284785809586792E-3</v>
       </c>
       <c r="D8">
-        <v>-1.9699348699017529</v>
+        <v>1.595454316306282</v>
       </c>
       <c r="E8">
-        <v>4.8845835442129608E-2</v>
+        <v>0.11061067804716621</v>
       </c>
       <c r="F8">
-        <v>-1.8314902578552979E-3</v>
+        <v>-4.6831684920394049E-4</v>
       </c>
       <c r="G8">
-        <v>-4.6468319105729501E-6</v>
+        <v>4.5679509800725564E-3</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -2585,22 +2585,22 @@
         <v>13</v>
       </c>
       <c r="B9">
-        <v>-1.054779922392548E-3</v>
+        <v>8.9783131402882332E-4</v>
       </c>
       <c r="C9">
-        <v>5.5522439136449322E-4</v>
+        <v>1.42633323930559E-3</v>
       </c>
       <c r="D9">
-        <v>-1.8997362846404691</v>
+        <v>0.62946812798524743</v>
       </c>
       <c r="E9">
-        <v>5.7467736099696187E-2</v>
+        <v>0.52904262827403514</v>
       </c>
       <c r="F9">
-        <v>-2.1429997328051261E-3</v>
+        <v>-1.897730464962482E-3</v>
       </c>
       <c r="G9">
-        <v>3.3439888020030681E-5</v>
+        <v>3.693393093020129E-3</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
@@ -2608,22 +2608,22 @@
         <v>14</v>
       </c>
       <c r="B10">
-        <v>-6.3054538991194425E-4</v>
+        <v>2.420968692152164E-3</v>
       </c>
       <c r="C10">
-        <v>3.252973429877047E-4</v>
+        <v>2.047194761741433E-3</v>
       </c>
       <c r="D10">
-        <v>-1.9383662470792979</v>
+        <v>1.182578588708767</v>
       </c>
       <c r="E10">
-        <v>5.257855532062778E-2</v>
+        <v>0.2369762023468904</v>
       </c>
       <c r="F10">
-        <v>-1.268116466434419E-3</v>
+        <v>-1.591459310200101E-3</v>
       </c>
       <c r="G10">
-        <v>7.0256866105300637E-6</v>
+        <v>6.4333966945044297E-3</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -2631,22 +2631,22 @@
         <v>15</v>
       </c>
       <c r="B11">
-        <v>9.5147445049984544E-4</v>
+        <v>1.1590503065176669E-3</v>
       </c>
       <c r="C11">
-        <v>7.5102069491487925E-4</v>
+        <v>9.4891782921007167E-4</v>
       </c>
       <c r="D11">
-        <v>1.26690843134181</v>
+        <v>1.2214443346296071</v>
       </c>
       <c r="E11">
-        <v>0.2051880336119585</v>
+        <v>0.22191782970437529</v>
       </c>
       <c r="F11">
-        <v>-5.2049906317756171E-4</v>
+        <v>-7.0079446302200336E-4</v>
       </c>
       <c r="G11">
-        <v>2.4234479641772519E-3</v>
+        <v>3.0188950760573381E-3</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
@@ -2654,22 +2654,22 @@
         <v>16</v>
       </c>
       <c r="B12">
-        <v>-3.0750188111641432E-5</v>
+        <v>1.12552168666992E-4</v>
       </c>
       <c r="C12">
-        <v>7.4833339489696301E-4</v>
+        <v>6.3408478701954506E-4</v>
       </c>
       <c r="D12">
-        <v>-4.1091562024804983E-2</v>
+        <v>0.17750334177868021</v>
       </c>
       <c r="E12">
-        <v>0.96722290145239187</v>
+        <v>0.85911304055429705</v>
       </c>
       <c r="F12">
-        <v>-1.497456690538279E-3</v>
+        <v>-1.130231177036067E-3</v>
       </c>
       <c r="G12">
-        <v>1.4359563143149961E-3</v>
+        <v>1.3553355143700509E-3</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
@@ -2677,22 +2677,22 @@
         <v>17</v>
       </c>
       <c r="B13">
-        <v>1.6381588681083799E-3</v>
+        <v>5.0106175847336818E-3</v>
       </c>
       <c r="C13">
-        <v>1.4597926672667611E-3</v>
+        <v>3.1060050734967128E-3</v>
       </c>
       <c r="D13">
-        <v>1.1221859821885409</v>
+        <v>1.613203284015494</v>
       </c>
       <c r="E13">
-        <v>0.26178337150972808</v>
+        <v>0.10670035022260239</v>
       </c>
       <c r="F13">
-        <v>-1.2229821846301331E-3</v>
+        <v>-1.077040495118559E-3</v>
       </c>
       <c r="G13">
-        <v>4.4992999208468944E-3</v>
+        <v>1.109827566458592E-2</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
@@ -2700,22 +2700,22 @@
         <v>18</v>
       </c>
       <c r="B14">
-        <v>1.538581864557001E-4</v>
+        <v>-3.0374733265739729E-3</v>
       </c>
       <c r="C14">
-        <v>8.7303713763912732E-4</v>
+        <v>2.3545216056226098E-3</v>
       </c>
       <c r="D14">
-        <v>0.17623326640120299</v>
+        <v>-1.2900596534431761</v>
       </c>
       <c r="E14">
-        <v>0.86011068696314952</v>
+        <v>0.197029946952855</v>
       </c>
       <c r="F14">
-        <v>-1.557263160482927E-3</v>
+        <v>-7.6522508744157093E-3</v>
       </c>
       <c r="G14">
-        <v>1.864979533394328E-3</v>
+        <v>1.5773042212677631E-3</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
@@ -2723,22 +2723,22 @@
         <v>19</v>
       </c>
       <c r="B15">
-        <v>-2.5855963956699811E-5</v>
+        <v>-2.1460767677695509E-3</v>
       </c>
       <c r="C15">
-        <v>6.5437927919359074E-4</v>
+        <v>1.8991273857780189E-3</v>
       </c>
       <c r="D15">
-        <v>-3.951219847389241E-2</v>
+        <v>-1.1300330793188811</v>
       </c>
       <c r="E15">
-        <v>0.96848202813652717</v>
+        <v>0.25846228607144722</v>
       </c>
       <c r="F15">
-        <v>-1.3084157834054181E-3</v>
+        <v>-5.8682980459481733E-3</v>
       </c>
       <c r="G15">
-        <v>1.2567038554920191E-3</v>
+        <v>1.5761445104090709E-3</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
@@ -2746,22 +2746,22 @@
         <v>20</v>
       </c>
       <c r="B16">
-        <v>3.356511398637704E-3</v>
+        <v>7.2716604597848405E-4</v>
       </c>
       <c r="C16">
-        <v>2.3449635773846911E-3</v>
+        <v>8.412814246176886E-4</v>
       </c>
       <c r="D16">
-        <v>1.4313703764990591</v>
+        <v>0.86435528552046292</v>
       </c>
       <c r="E16">
-        <v>0.15232409379086029</v>
+        <v>0.38739274828046127</v>
       </c>
       <c r="F16">
-        <v>-1.2395327580944941E-3</v>
+        <v>-9.2171524713473394E-4</v>
       </c>
       <c r="G16">
-        <v>7.9525555553699029E-3</v>
+        <v>2.3760473390917018E-3</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
@@ -2769,22 +2769,22 @@
         <v>21</v>
       </c>
       <c r="B17">
-        <v>-2.7703729394140939E-3</v>
+        <v>6.1735910943654625E-4</v>
       </c>
       <c r="C17">
-        <v>1.654670601266017E-3</v>
+        <v>7.5430221833843174E-4</v>
       </c>
       <c r="D17">
-        <v>-1.6742745881231189</v>
+        <v>0.81845060829392469</v>
       </c>
       <c r="E17">
-        <v>9.4076646365648317E-2</v>
+        <v>0.41309993409035528</v>
       </c>
       <c r="F17">
-        <v>-6.013467724172725E-3</v>
+        <v>-8.6104607196544822E-4</v>
       </c>
       <c r="G17">
-        <v>4.7272184534453629E-4</v>
+        <v>2.0957642908385411E-3</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
@@ -2792,22 +2792,22 @@
         <v>22</v>
       </c>
       <c r="B18">
-        <v>-8.0985230215565999E-4</v>
+        <v>8.1215789987781721E-4</v>
       </c>
       <c r="C18">
-        <v>4.8086360158022953E-4</v>
+        <v>9.8645397938355254E-4</v>
       </c>
       <c r="D18">
-        <v>-1.6841622021178091</v>
+        <v>0.82331048062206091</v>
       </c>
       <c r="E18">
-        <v>9.2150325852993958E-2</v>
+        <v>0.41033145512365748</v>
       </c>
       <c r="F18">
-        <v>-1.752327642729127E-3</v>
+        <v>-1.121256372120163E-3</v>
       </c>
       <c r="G18">
-        <v>1.326230384178076E-4</v>
+        <v>2.745572171875797E-3</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
@@ -2815,22 +2815,22 @@
         <v>23</v>
       </c>
       <c r="B19">
-        <v>-5.588583314536477E-4</v>
+        <v>3.9026510206130292E-4</v>
       </c>
       <c r="C19">
-        <v>6.8302265319579707E-4</v>
+        <v>7.5595522597380108E-4</v>
       </c>
       <c r="D19">
-        <v>-0.81821346457369093</v>
+        <v>0.51625425508312861</v>
       </c>
       <c r="E19">
-        <v>0.41323530809564513</v>
+        <v>0.60567684131968247</v>
       </c>
       <c r="F19">
-        <v>-1.8975581323424019E-3</v>
+        <v>-1.091379914772185E-3</v>
       </c>
       <c r="G19">
-        <v>7.7984146943510611E-4</v>
+        <v>1.871910118894791E-3</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
@@ -2838,22 +2838,22 @@
         <v>24</v>
       </c>
       <c r="B20">
-        <v>-1.5468261191417709E-3</v>
+        <v>9.6386200479331788E-4</v>
       </c>
       <c r="C20">
-        <v>6.6683577109437103E-4</v>
+        <v>9.9366968146097768E-4</v>
       </c>
       <c r="D20">
-        <v>-2.319650783885232</v>
+        <v>0.97000242915348489</v>
       </c>
       <c r="E20">
-        <v>2.035977625626894E-2</v>
+        <v>0.33204528130404459</v>
       </c>
       <c r="F20">
-        <v>-2.853800214089733E-3</v>
+        <v>-9.8369478339958632E-4</v>
       </c>
       <c r="G20">
-        <v>-2.3985202419380761E-4</v>
+        <v>2.9114187929862221E-3</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
@@ -2861,22 +2861,22 @@
         <v>25</v>
       </c>
       <c r="B21">
-        <v>0.38779864034482309</v>
+        <v>0.47807043465310139</v>
       </c>
       <c r="C21">
-        <v>0.1165945463908795</v>
+        <v>7.3171531340017706E-2</v>
       </c>
       <c r="D21">
-        <v>3.3260444193053469</v>
+        <v>6.5335578728231889</v>
       </c>
       <c r="E21">
-        <v>8.8087889589230813E-4</v>
+        <v>6.4225359648525417E-11</v>
       </c>
       <c r="F21">
-        <v>0.15927752862491479</v>
+        <v>0.33465686853302279</v>
       </c>
       <c r="G21">
-        <v>0.61631975206473144</v>
+        <v>0.62148400077317989</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
@@ -2884,22 +2884,22 @@
         <v>26</v>
       </c>
       <c r="B22">
-        <v>0.1480607362023533</v>
+        <v>0.45091844266107539</v>
       </c>
       <c r="C22">
-        <v>8.7418737697163754E-2</v>
+        <v>5.6614173702536831E-2</v>
       </c>
       <c r="D22">
-        <v>1.693695654989503</v>
+        <v>7.9647624114466256</v>
       </c>
       <c r="E22">
-        <v>9.0323130553848371E-2</v>
+        <v>1.655415305708788E-15</v>
       </c>
       <c r="F22">
-        <v>-2.3276841258041581E-2</v>
+        <v>0.33995670118960858</v>
       </c>
       <c r="G22">
-        <v>0.31939831366274818</v>
+        <v>0.56188018413254226</v>
       </c>
     </row>
   </sheetData>
@@ -2937,22 +2937,22 @@
         <v>6</v>
       </c>
       <c r="B2">
-        <v>1.2472243333431989E-4</v>
+        <v>4.5610218047794282E-3</v>
       </c>
       <c r="C2">
-        <v>7.8409232616590452E-4</v>
+        <v>1.734949086520048E-3</v>
       </c>
       <c r="D2">
-        <v>0.15906600431124501</v>
+        <v>2.6289081565660819</v>
       </c>
       <c r="E2">
-        <v>0.87361687179061542</v>
+        <v>8.5659492055551421E-3</v>
       </c>
       <c r="F2">
-        <v>-1.412070286505086E-3</v>
+        <v>1.160584080189468E-3</v>
       </c>
       <c r="G2">
-        <v>1.661515153173726E-3</v>
+        <v>7.9614595293693892E-3</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -2960,22 +2960,22 @@
         <v>7</v>
       </c>
       <c r="B3">
-        <v>2.392222769270902E-3</v>
+        <v>-2.6600600890392609E-3</v>
       </c>
       <c r="C3">
-        <v>3.93414772656941E-4</v>
+        <v>5.107454112740586E-3</v>
       </c>
       <c r="D3">
-        <v>6.0806632987239846</v>
+        <v>-0.52081918512076675</v>
       </c>
       <c r="E3">
-        <v>1.1968638734941939E-9</v>
+        <v>0.60249273698585637</v>
       </c>
       <c r="F3">
-        <v>1.6211439838772839E-3</v>
+        <v>-1.2670486202701789E-2</v>
       </c>
       <c r="G3">
-        <v>3.163301554664519E-3</v>
+        <v>7.350366024623264E-3</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
@@ -2983,22 +2983,22 @@
         <v>8</v>
       </c>
       <c r="B4">
-        <v>-1.6092108607047269E-3</v>
+        <v>-2.1648699559862969E-3</v>
       </c>
       <c r="C4">
-        <v>7.6452729192480072E-4</v>
+        <v>5.2040215598236116E-3</v>
       </c>
       <c r="D4">
-        <v>-2.1048442321180212</v>
+        <v>-0.41599942104384252</v>
       </c>
       <c r="E4">
-        <v>3.5304869455762757E-2</v>
+        <v>0.67741042686564246</v>
       </c>
       <c r="F4">
-        <v>-3.1076568180752758E-3</v>
+        <v>-1.236456478801053E-2</v>
       </c>
       <c r="G4">
-        <v>-1.107649033341774E-4</v>
+        <v>8.0348248760379378E-3</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -3006,22 +3006,22 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>2.6236206493700899E-3</v>
+        <v>1.573269020307036E-3</v>
       </c>
       <c r="C5">
-        <v>3.5337282028657991E-3</v>
+        <v>2.773770251720196E-3</v>
       </c>
       <c r="D5">
-        <v>0.74245117302524111</v>
+        <v>0.5671951450670254</v>
       </c>
       <c r="E5">
-        <v>0.45781402464516358</v>
+        <v>0.57058160615024511</v>
       </c>
       <c r="F5">
-        <v>-4.3023593594003259E-3</v>
+        <v>-3.863220774453148E-3</v>
       </c>
       <c r="G5">
-        <v>9.549600658140504E-3</v>
+        <v>7.0097588150672199E-3</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -3029,22 +3029,22 @@
         <v>10</v>
       </c>
       <c r="B6">
-        <v>-7.294975838405225E-3</v>
+        <v>2.404344531488762E-3</v>
       </c>
       <c r="C6">
-        <v>2.365166595099511E-3</v>
+        <v>2.6993660355725899E-3</v>
       </c>
       <c r="D6">
-        <v>-3.0843391131601439</v>
+        <v>0.890707114116427</v>
       </c>
       <c r="E6">
-        <v>2.040049160120893E-3</v>
+        <v>0.37308631723433039</v>
       </c>
       <c r="F6">
-        <v>-1.19306171822375E-2</v>
+        <v>-2.8863156793241811E-3</v>
       </c>
       <c r="G6">
-        <v>-2.6593344945729539E-3</v>
+        <v>7.6950047423017054E-3</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
@@ -3052,22 +3052,22 @@
         <v>11</v>
       </c>
       <c r="B7">
-        <v>-4.8019696355746846E-3</v>
+        <v>1.1836001136659789E-3</v>
       </c>
       <c r="C7">
-        <v>1.075126414817852E-3</v>
+        <v>3.1051238133401279E-3</v>
       </c>
       <c r="D7">
-        <v>-4.466423268363501</v>
+        <v>0.38117646342507722</v>
       </c>
       <c r="E7">
-        <v>7.9538171347471073E-6</v>
+        <v>0.70307231260227088</v>
       </c>
       <c r="F7">
-        <v>-6.9091786874453474E-3</v>
+        <v>-4.9023307280183451E-3</v>
       </c>
       <c r="G7">
-        <v>-2.694760583704024E-3</v>
+        <v>7.2695309553503038E-3</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
@@ -3075,22 +3075,22 @@
         <v>12</v>
       </c>
       <c r="B8">
-        <v>-3.9438035580385937E-3</v>
+        <v>5.5253983035709678E-3</v>
       </c>
       <c r="C8">
-        <v>9.2747540073365457E-4</v>
+        <v>2.8953611792987759E-3</v>
       </c>
       <c r="D8">
-        <v>-4.2521920850072723</v>
+        <v>1.90836236358918</v>
       </c>
       <c r="E8">
-        <v>2.1168816603699189E-5</v>
+        <v>5.634439774770536E-2</v>
       </c>
       <c r="F8">
-        <v>-5.7616219400234104E-3</v>
+        <v>-1.494053300900508E-4</v>
       </c>
       <c r="G8">
-        <v>-2.125985176053777E-3</v>
+        <v>1.120020193723199E-2</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -3098,22 +3098,22 @@
         <v>13</v>
       </c>
       <c r="B9">
-        <v>-3.3647489011615641E-3</v>
+        <v>7.0511992134935867E-3</v>
       </c>
       <c r="C9">
-        <v>9.7813052339774964E-4</v>
+        <v>4.8025630053679866E-3</v>
       </c>
       <c r="D9">
-        <v>-3.4399794512836328</v>
+        <v>1.4682158684044799</v>
       </c>
       <c r="E9">
-        <v>5.8175835445783226E-4</v>
+        <v>0.14204559521280211</v>
       </c>
       <c r="F9">
-        <v>-5.2818494992004656E-3</v>
+        <v>-2.361651310512108E-3</v>
       </c>
       <c r="G9">
-        <v>-1.4476483031226619E-3</v>
+        <v>1.6464049737499278E-2</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
@@ -3121,22 +3121,22 @@
         <v>14</v>
       </c>
       <c r="B10">
-        <v>-4.5071644565110817E-3</v>
+        <v>2.523791446544132E-3</v>
       </c>
       <c r="C10">
-        <v>1.064761204428738E-3</v>
+        <v>1.1450802538672261E-2</v>
       </c>
       <c r="D10">
-        <v>-4.2330284365772419</v>
+        <v>0.22040301874219281</v>
       </c>
       <c r="E10">
-        <v>2.305653385801423E-5</v>
+        <v>0.8255572946001577</v>
       </c>
       <c r="F10">
-        <v>-6.5940580693268983E-3</v>
+        <v>-1.9919369123333329E-2</v>
       </c>
       <c r="G10">
-        <v>-2.4202708436952651E-3</v>
+        <v>2.496695201642159E-2</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -3144,22 +3144,22 @@
         <v>15</v>
       </c>
       <c r="B11">
-        <v>-1.565038838011066E-4</v>
+        <v>6.7964937062316606E-3</v>
       </c>
       <c r="C11">
-        <v>9.271597159261029E-4</v>
+        <v>4.5165790131534928E-3</v>
       </c>
       <c r="D11">
-        <v>-0.16879927062489031</v>
+        <v>1.504787957088416</v>
       </c>
       <c r="E11">
-        <v>0.86595453205004258</v>
+        <v>0.13237860092312559</v>
       </c>
       <c r="F11">
-        <v>-1.9737035349326562E-3</v>
+        <v>-2.055838492878645E-3</v>
       </c>
       <c r="G11">
-        <v>1.6606957673304429E-3</v>
+        <v>1.564882590534197E-2</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
@@ -3167,22 +3167,22 @@
         <v>16</v>
       </c>
       <c r="B12">
-        <v>3.573811610374282E-3</v>
+        <v>1.09842303528714E-2</v>
       </c>
       <c r="C12">
-        <v>3.7149316791137972E-3</v>
+        <v>7.0213780346768664E-3</v>
       </c>
       <c r="D12">
-        <v>0.96201274184046925</v>
+        <v>1.564398085193957</v>
       </c>
       <c r="E12">
-        <v>0.33604320346423411</v>
+        <v>0.11772411011702739</v>
       </c>
       <c r="F12">
-        <v>-3.7073206857156692E-3</v>
+        <v>-2.777417716935886E-3</v>
       </c>
       <c r="G12">
-        <v>1.0854943906464231E-2</v>
+        <v>2.4745878422678679E-2</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
@@ -3190,22 +3190,22 @@
         <v>17</v>
       </c>
       <c r="B13">
-        <v>6.2407269962541027E-4</v>
+        <v>7.5361562133257516E-3</v>
       </c>
       <c r="C13">
-        <v>4.8532381544080551E-3</v>
+        <v>7.6956606414042379E-3</v>
       </c>
       <c r="D13">
-        <v>0.12858892965278931</v>
+        <v>0.97927345870472515</v>
       </c>
       <c r="E13">
-        <v>0.89768292643639502</v>
+        <v>0.32744488090383489</v>
       </c>
       <c r="F13">
-        <v>-8.8880992914100194E-3</v>
+        <v>-7.5470614810689667E-3</v>
       </c>
       <c r="G13">
-        <v>1.013624469066084E-2</v>
+        <v>2.261937390772047E-2</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
@@ -3213,22 +3213,22 @@
         <v>18</v>
       </c>
       <c r="B14">
-        <v>5.8121257945539947E-4</v>
+        <v>-1.0508454088332279E-2</v>
       </c>
       <c r="C14">
-        <v>3.1381462412703692E-3</v>
+        <v>5.5134824649988494E-3</v>
       </c>
       <c r="D14">
-        <v>0.1852088891880691</v>
+        <v>-1.905955837357411</v>
       </c>
       <c r="E14">
-        <v>0.85306519714827411</v>
+        <v>5.6655935633805103E-2</v>
       </c>
       <c r="F14">
-        <v>-5.5694410316542674E-3</v>
+        <v>-2.131468114912315E-2</v>
       </c>
       <c r="G14">
-        <v>6.7318661905650667E-3</v>
+        <v>2.9777297245857891E-4</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
@@ -3236,22 +3236,22 @@
         <v>19</v>
       </c>
       <c r="B15">
-        <v>6.7227995844211822E-3</v>
+        <v>-4.2857097858217223E-3</v>
       </c>
       <c r="C15">
-        <v>5.3935133084345851E-3</v>
+        <v>7.0172316047516173E-3</v>
       </c>
       <c r="D15">
-        <v>1.2464601828103039</v>
+        <v>-0.61074082020033593</v>
       </c>
       <c r="E15">
-        <v>0.21259549840380959</v>
+        <v>0.54137117742573582</v>
       </c>
       <c r="F15">
-        <v>-3.8482922502480759E-3</v>
+        <v>-1.8039231002311099E-2</v>
       </c>
       <c r="G15">
-        <v>1.7293891419090442E-2</v>
+        <v>9.4678114306676556E-3</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
@@ -3259,22 +3259,22 @@
         <v>20</v>
       </c>
       <c r="B16">
-        <v>4.5777881088040623E-3</v>
+        <v>3.2398023656409632E-3</v>
       </c>
       <c r="C16">
-        <v>6.2927810347581329E-3</v>
+        <v>2.732780314803473E-3</v>
       </c>
       <c r="D16">
-        <v>0.72746661349229869</v>
+        <v>1.1855334100918939</v>
       </c>
       <c r="E16">
-        <v>0.46694016045782533</v>
+        <v>0.23580661301112349</v>
       </c>
       <c r="F16">
-        <v>-7.7558360819185729E-3</v>
+        <v>-2.1163486290338759E-3</v>
       </c>
       <c r="G16">
-        <v>1.6911412299526699E-2</v>
+        <v>8.5959533603158014E-3</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
@@ -3282,22 +3282,22 @@
         <v>21</v>
       </c>
       <c r="B17">
-        <v>-7.1221378337270906E-3</v>
+        <v>3.486975878344685E-3</v>
       </c>
       <c r="C17">
-        <v>3.256832210306313E-3</v>
+        <v>2.8157058314056821E-3</v>
       </c>
       <c r="D17">
-        <v>-2.1868298315120249</v>
+        <v>1.2384020516105849</v>
       </c>
       <c r="E17">
-        <v>2.8754948855740561E-2</v>
+        <v>0.21556702030506489</v>
       </c>
       <c r="F17">
-        <v>-1.350541166961744E-2</v>
+        <v>-2.0317061422698611E-3</v>
       </c>
       <c r="G17">
-        <v>-7.3886399783673791E-4</v>
+        <v>9.0056578989592302E-3</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
@@ -3305,22 +3305,22 @@
         <v>22</v>
       </c>
       <c r="B18">
-        <v>-1.351989323774022E-3</v>
+        <v>3.2487335470471508E-3</v>
       </c>
       <c r="C18">
-        <v>2.4205683826192632E-3</v>
+        <v>2.3828650503622262E-3</v>
       </c>
       <c r="D18">
-        <v>-0.55854209014787426</v>
+        <v>1.3633728635003071</v>
       </c>
       <c r="E18">
-        <v>0.5764742714267973</v>
+        <v>0.17276502892908141</v>
       </c>
       <c r="F18">
-        <v>-6.0962161758241467E-3</v>
+        <v>-1.4215961316820351E-3</v>
       </c>
       <c r="G18">
-        <v>3.3922375282761019E-3</v>
+        <v>7.9190632257763356E-3</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
@@ -3328,22 +3328,22 @@
         <v>23</v>
       </c>
       <c r="B19">
-        <v>-2.327952030786477E-3</v>
+        <v>5.0830946164571317E-3</v>
       </c>
       <c r="C19">
-        <v>3.9466394793509487E-3</v>
+        <v>2.9648836583874732E-3</v>
       </c>
       <c r="D19">
-        <v>-0.58985677383669299</v>
+        <v>1.714433078032378</v>
       </c>
       <c r="E19">
-        <v>0.55528667616474037</v>
+        <v>8.644921788554695E-2</v>
       </c>
       <c r="F19">
-        <v>-1.0063223270278251E-2</v>
+        <v>-7.2797057233367317E-4</v>
       </c>
       <c r="G19">
-        <v>5.4073192087052933E-3</v>
+        <v>1.089415980524794E-2</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
@@ -3351,22 +3351,22 @@
         <v>24</v>
       </c>
       <c r="B20">
-        <v>-2.7569099893735289E-3</v>
+        <v>4.4992561106867932E-3</v>
       </c>
       <c r="C20">
-        <v>3.3000678968588019E-3</v>
+        <v>2.8971069269304261E-3</v>
       </c>
       <c r="D20">
-        <v>-0.83541008110703341</v>
+        <v>1.553016931775415</v>
       </c>
       <c r="E20">
-        <v>0.40348685567473191</v>
+        <v>0.120419089603835</v>
       </c>
       <c r="F20">
-        <v>-9.2249242137536231E-3</v>
+        <v>-1.1789691254583559E-3</v>
       </c>
       <c r="G20">
-        <v>3.7111042350065652E-3</v>
+        <v>1.017748134683194E-2</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
@@ -3374,22 +3374,22 @@
         <v>25</v>
       </c>
       <c r="B21">
-        <v>0.24428960410750669</v>
+        <v>0.46687358440536941</v>
       </c>
       <c r="C21">
-        <v>0.1008107381370818</v>
+        <v>5.6686388846750799E-2</v>
       </c>
       <c r="D21">
-        <v>2.4232498305420931</v>
+        <v>8.236079134755645</v>
       </c>
       <c r="E21">
-        <v>1.5382343941073569E-2</v>
+        <v>1.7794625507685011E-16</v>
       </c>
       <c r="F21">
-        <v>4.6704188103927902E-2</v>
+        <v>0.35577030385210479</v>
       </c>
       <c r="G21">
-        <v>0.44187502011108548</v>
+        <v>0.57797686495863387</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
@@ -3397,22 +3397,22 @@
         <v>26</v>
       </c>
       <c r="B22">
-        <v>0.23035631863386499</v>
+        <v>0.50872055476944411</v>
       </c>
       <c r="C22">
-        <v>3.5834189815554147E-2</v>
+        <v>5.2477456685249287E-2</v>
       </c>
       <c r="D22">
-        <v>6.428394776596198</v>
+        <v>9.6940779317995922</v>
       </c>
       <c r="E22">
-        <v>1.2895847220808761E-10</v>
+        <v>3.195105749370884E-22</v>
       </c>
       <c r="F22">
-        <v>0.1601225971802068</v>
+        <v>0.40586662966609482</v>
       </c>
       <c r="G22">
-        <v>0.30059004008752321</v>
+        <v>0.61157447987279334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>